<commit_message>
systeem om taal te wisselen tussen fr/nl gemaakt
</commit_message>
<xml_diff>
--- a/Planning week project.xlsx
+++ b/Planning week project.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ehb-my.sharepoint.com/personal/lilian_levano_student_ehb_be/Documents/école ehb/cours/dynamic web prg1 s2/ExamenProject/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ehb-my.sharepoint.com/personal/lilian_levano_student_ehb_be/Documents/école ehb/cours/dynamic web prg1 s2/ExamenProject/Project-Dynamic-Web/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="64" documentId="11_F25DC773A252ABDACC10483A31DF42745BDE58EE" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F48EB10B-A649-4C83-B57E-57EFFA178498}"/>
+  <xr:revisionPtr revIDLastSave="78" documentId="11_F25DC773A252ABDACC10483A31DF42745BDE58EE" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{685F6D58-C6C2-40AD-9769-553C878EEECF}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
   <si>
     <t>Mardi</t>
   </si>
@@ -67,7 +67,28 @@
   <si>
     <t>Verwerk data in de lijst
 Zoekmethode (aanleggen classe in CSS)
-LocalStorage</t>
+systeem van favoriete locaties (localstorage)</t>
+  </si>
+  <si>
+    <t>mogelijkheid om van thema te switchen (+ localstorage)
+formulier validatie? (niet zeker wat het is, moet vragen)</t>
+  </si>
+  <si>
+    <t>resposive design (als niet genoeg tijd op woensdag)
+sorteer mogelijkheid</t>
+  </si>
+  <si>
+    <t xml:space="preserve">commentaar toevoegen waar nodig
+backlog en user stories afwerken
+readme(
+- ProjectBeschrijving + Functionaliteiten opsommen
+- Link naar API
+-Documenteren van elke technisch verseiste (tabel met: vereiste | hoe | lijn code)
+-Installatiehandleiding (repo clone --&gt; index.html)
+-Screenshots van app
+- Gebruikte bronnen (AI, etc)
+- Taak verdeling)
+</t>
   </si>
 </sst>
 </file>
@@ -177,10 +198,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -495,13 +512,19 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="93.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" ht="409.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="4"/>
-      <c r="C4" s="4"/>
-      <c r="D4" s="4"/>
+      <c r="B4" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="5" spans="1:4" ht="151.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">

</xml_diff>

<commit_message>
aanpassingen user stories en backlog
</commit_message>
<xml_diff>
--- a/Planning week project.xlsx
+++ b/Planning week project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ehb-my.sharepoint.com/personal/lilian_levano_student_ehb_be/Documents/école ehb/cours/dynamic web prg1 s2/ExamenProject/Project-Dynamic-Web/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="78" documentId="11_F25DC773A252ABDACC10483A31DF42745BDE58EE" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{685F6D58-C6C2-40AD-9769-553C878EEECF}"/>
+  <xr:revisionPtr revIDLastSave="81" documentId="11_F25DC773A252ABDACC10483A31DF42745BDE58EE" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{274E4DC4-3861-4397-AD05-14B268125620}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
   <si>
     <t>Mardi</t>
   </si>
@@ -63,15 +63,6 @@
     <t>Fetch API, omzetten naar JSON
 Filtreer optie
 Responsive design</t>
-  </si>
-  <si>
-    <t>Verwerk data in de lijst
-Zoekmethode (aanleggen classe in CSS)
-systeem van favoriete locaties (localstorage)</t>
-  </si>
-  <si>
-    <t>mogelijkheid om van thema te switchen (+ localstorage)
-formulier validatie? (niet zeker wat het is, moet vragen)</t>
   </si>
   <si>
     <t>resposive design (als niet genoeg tijd op woensdag)
@@ -89,6 +80,19 @@
 - Gebruikte bronnen (AI, etc)
 - Taak verdeling)
 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verwerk data in de lijst
+Zoekmethode (aanleggen classe in CSS)
+</t>
+  </si>
+  <si>
+    <t>mogelijkheid om van thema te switchen (+ localstorage)
+systeem van favoriete locaties (localstorage)
+formulier validatie? (niet zeker wat het is, moet vragen)</t>
+  </si>
+  <si>
+    <t>readme verder bouwen (afmaken)</t>
   </si>
 </sst>
 </file>
@@ -198,6 +202,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -503,7 +511,7 @@
         <v>1</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C3" s="6" t="s">
         <v>11</v>
@@ -517,13 +525,13 @@
         <v>2</v>
       </c>
       <c r="B4" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="D4" s="6" t="s">
         <v>13</v>
-      </c>
-      <c r="C4" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="D4" s="6" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="151.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -532,7 +540,9 @@
       </c>
       <c r="B5" s="4"/>
       <c r="C5" s="4"/>
-      <c r="D5" s="4"/>
+      <c r="D5" s="4" t="s">
+        <v>16</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
aanpassingen user story en backlog aangepast + kleine fout in js aangepast
</commit_message>
<xml_diff>
--- a/Planning week project.xlsx
+++ b/Planning week project.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ehb-my.sharepoint.com/personal/lilian_levano_student_ehb_be/Documents/école ehb/cours/dynamic web prg1 s2/ExamenProject/Project-Dynamic-Web/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="81" documentId="11_F25DC773A252ABDACC10483A31DF42745BDE58EE" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{274E4DC4-3861-4397-AD05-14B268125620}"/>
+  <xr:revisionPtr revIDLastSave="85" documentId="11_F25DC773A252ABDACC10483A31DF42745BDE58EE" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FBDDDB29-782C-4777-8F99-DC0DCF242F76}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -65,10 +65,6 @@
 Responsive design</t>
   </si>
   <si>
-    <t>resposive design (als niet genoeg tijd op woensdag)
-sorteer mogelijkheid</t>
-  </si>
-  <si>
     <t xml:space="preserve">commentaar toevoegen waar nodig
 backlog en user stories afwerken
 readme(
@@ -87,12 +83,17 @@
 </t>
   </si>
   <si>
-    <t>mogelijkheid om van thema te switchen (+ localstorage)
-systeem van favoriete locaties (localstorage)
-formulier validatie? (niet zeker wat het is, moet vragen)</t>
-  </si>
-  <si>
     <t>readme verder bouwen (afmaken)</t>
+  </si>
+  <si>
+    <t>resposive design (als niet genoeg tijd op woensdag)
+sorteer mogelijkheid
+voeg foutmeldingen wanneer er geen resultaat gevonden werd voor de verschillende filteer / zoek opties</t>
+  </si>
+  <si>
+    <t xml:space="preserve">systeem van favoriete locaties (localstorage)
+formulier validatie voor input filter 
+</t>
   </si>
 </sst>
 </file>
@@ -511,7 +512,7 @@
         <v>1</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C3" s="6" t="s">
         <v>11</v>
@@ -525,13 +526,13 @@
         <v>2</v>
       </c>
       <c r="B4" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="C4" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="D4" s="6" t="s">
         <v>12</v>
-      </c>
-      <c r="D4" s="6" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="151.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -541,7 +542,7 @@
       <c r="B5" s="4"/>
       <c r="C5" s="4"/>
       <c r="D5" s="4" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
sorteer methode van de locacationnaam alfabetisch voor filter search aan gemaakt en backlog gewijzigd
</commit_message>
<xml_diff>
--- a/Planning week project.xlsx
+++ b/Planning week project.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ehb-my.sharepoint.com/personal/lilian_levano_student_ehb_be/Documents/école ehb/cours/dynamic web prg1 s2/ExamenProject/Project-Dynamic-Web/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bilal\Desktop\ehb_vakken\dynamicWeb\Exam\Project-Dynamic-Web\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="81" documentId="11_F25DC773A252ABDACC10483A31DF42745BDE58EE" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{274E4DC4-3861-4397-AD05-14B268125620}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -202,10 +202,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>

<commit_message>
backlog / US aangepast
</commit_message>
<xml_diff>
--- a/Planning week project.xlsx
+++ b/Planning week project.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bilal\Desktop\ehb_vakken\dynamicWeb\Exam\Project-Dynamic-Web\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ehb-my.sharepoint.com/personal/lilian_levano_student_ehb_be/Documents/école ehb/cours/dynamic web prg1 s2/ExamenProject/Project-Dynamic-Web/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="81" documentId="11_F25DC773A252ABDACC10483A31DF42745BDE58EE" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{274E4DC4-3861-4397-AD05-14B268125620}"/>
+  <xr:revisionPtr revIDLastSave="86" documentId="11_F25DC773A252ABDACC10483A31DF42745BDE58EE" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C8D619EF-E49F-594E-95F6-F45E4CC13F18}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>